<commit_message>
agora vai esse cache
</commit_message>
<xml_diff>
--- a/saidas/comparativo_marco_qtd_4_b_top_5.xlsx
+++ b/saidas/comparativo_marco_qtd_4_b_top_5.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>Dia Previsto</t>
   </si>
@@ -22,31 +22,58 @@
     <t>Realizado</t>
   </si>
   <si>
+    <t>Previsto_SE(LINE)+SE(SGDR)+ABR</t>
+  </si>
+  <si>
+    <t>Vies_SE(LINE)+SE(SGDR)+ABR</t>
+  </si>
+  <si>
+    <t>Previsto_SPct+ABR</t>
+  </si>
+  <si>
+    <t>Vies_SPct+ABR</t>
+  </si>
+  <si>
     <t>Previsto_SARIMA</t>
   </si>
   <si>
     <t>Vies_SARIMA</t>
   </si>
   <si>
-    <t>Previsto_SE(LINE)+SE(SGDR)+ABR</t>
-  </si>
-  <si>
-    <t>Vies_SE(LINE)+SE(SGDR)+ABR</t>
-  </si>
-  <si>
     <t>Previsto_Pipeline Antiga em Producao</t>
   </si>
   <si>
     <t>Vies_Pipeline Antiga em Producao</t>
   </si>
   <si>
+    <t>Previsto_SE(ABR)+MAS+OHE+ABR</t>
+  </si>
+  <si>
+    <t>Vies_SE(ABR)+MAS+OHE+ABR</t>
+  </si>
+  <si>
+    <t>Previsto_SE(ETR)+MMS+BIN+SE(ELAS)+ABR</t>
+  </si>
+  <si>
+    <t>Vies_SE(ETR)+MMS+BIN+SE(ELAS)+ABR</t>
+  </si>
+  <si>
     <t>Melhor Previsao</t>
   </si>
   <si>
+    <t>SPct+ABR</t>
+  </si>
+  <si>
+    <t>SE(ABR)+MAS+OHE+ABR</t>
+  </si>
+  <si>
+    <t>Pipeline Antiga em Producao</t>
+  </si>
+  <si>
     <t>SE(LINE)+SE(SGDR)+ABR</t>
   </si>
   <si>
-    <t>Pipeline Antiga em Producao</t>
+    <t>SE(ETR)+MMS+BIN+SE(ELAS)+ABR</t>
   </si>
   <si>
     <t>SARIMA</t>
@@ -411,10 +438,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,8 +469,26 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" s="2">
         <v>46083</v>
       </c>
@@ -451,28 +496,46 @@
         <v>2844</v>
       </c>
       <c r="C2">
-        <v>3056.652387452421</v>
+        <v>2935.4</v>
       </c>
       <c r="D2">
-        <v>-212.6523874524214</v>
+        <v>-91.40000000000009</v>
       </c>
       <c r="E2">
-        <v>2935.4</v>
+        <v>2861.8</v>
       </c>
       <c r="F2">
-        <v>-91.40000000000009</v>
+        <v>-17.80000000000018</v>
       </c>
       <c r="G2">
+        <v>2983.812595969279</v>
+      </c>
+      <c r="H2">
+        <v>-139.8125959692788</v>
+      </c>
+      <c r="I2">
         <v>2996.3</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>-152.3000000000002</v>
       </c>
-      <c r="I2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="K2">
+        <v>2981</v>
+      </c>
+      <c r="L2">
+        <v>-137</v>
+      </c>
+      <c r="M2">
+        <v>2935.9</v>
+      </c>
+      <c r="N2">
+        <v>-91.90000000000009</v>
+      </c>
+      <c r="O2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="2">
         <v>46084</v>
       </c>
@@ -480,28 +543,46 @@
         <v>2487</v>
       </c>
       <c r="C3">
-        <v>2957.690265852616</v>
+        <v>2782.7</v>
       </c>
       <c r="D3">
-        <v>-470.6902658526155</v>
+        <v>-295.6999999999998</v>
       </c>
       <c r="E3">
-        <v>2782.7</v>
+        <v>2872.1</v>
       </c>
       <c r="F3">
-        <v>-295.6999999999998</v>
+        <v>-385.0999999999999</v>
       </c>
       <c r="G3">
+        <v>2893.341547827396</v>
+      </c>
+      <c r="H3">
+        <v>-406.3415478273964</v>
+      </c>
+      <c r="I3">
         <v>2970.3</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>-483.3000000000002</v>
       </c>
-      <c r="I3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="K3">
+        <v>2669</v>
+      </c>
+      <c r="L3">
+        <v>-182</v>
+      </c>
+      <c r="M3">
+        <v>2925.1</v>
+      </c>
+      <c r="N3">
+        <v>-438.0999999999999</v>
+      </c>
+      <c r="O3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="2">
         <v>46085</v>
       </c>
@@ -509,28 +590,46 @@
         <v>2680</v>
       </c>
       <c r="C4">
-        <v>2892.332028496444</v>
+        <v>2693.9</v>
       </c>
       <c r="D4">
-        <v>-212.3320284964443</v>
+        <v>-13.90000000000009</v>
       </c>
       <c r="E4">
-        <v>2693.9</v>
+        <v>2883.4</v>
       </c>
       <c r="F4">
-        <v>-13.90000000000009</v>
+        <v>-203.4000000000001</v>
       </c>
       <c r="G4">
+        <v>2777.504661920041</v>
+      </c>
+      <c r="H4">
+        <v>-97.50466192004114</v>
+      </c>
+      <c r="I4">
         <v>2678.8</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>1.199999999999818</v>
       </c>
-      <c r="I4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="K4">
+        <v>2623</v>
+      </c>
+      <c r="L4">
+        <v>57</v>
+      </c>
+      <c r="M4">
+        <v>2825.5</v>
+      </c>
+      <c r="N4">
+        <v>-145.5</v>
+      </c>
+      <c r="O4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="2">
         <v>46086</v>
       </c>
@@ -538,28 +637,46 @@
         <v>2608</v>
       </c>
       <c r="C5">
-        <v>2821.463280780648</v>
+        <v>2717.2</v>
       </c>
       <c r="D5">
-        <v>-213.4632807806479</v>
+        <v>-109.1999999999998</v>
       </c>
       <c r="E5">
-        <v>2717.2</v>
+        <v>2723.3</v>
       </c>
       <c r="F5">
-        <v>-109.1999999999998</v>
+        <v>-115.3000000000002</v>
       </c>
       <c r="G5">
+        <v>2720.553496018583</v>
+      </c>
+      <c r="H5">
+        <v>-112.5534960185828</v>
+      </c>
+      <c r="I5">
         <v>2807.3</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>-199.3000000000002</v>
       </c>
-      <c r="I5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="K5">
+        <v>2743.6</v>
+      </c>
+      <c r="L5">
+        <v>-135.5999999999999</v>
+      </c>
+      <c r="M5">
+        <v>2855.9</v>
+      </c>
+      <c r="N5">
+        <v>-247.9000000000001</v>
+      </c>
+      <c r="O5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="2">
         <v>46087</v>
       </c>
@@ -567,28 +684,46 @@
         <v>2715</v>
       </c>
       <c r="C6">
-        <v>2753.090898777894</v>
+        <v>2776.2</v>
       </c>
       <c r="D6">
-        <v>-38.09089877789393</v>
+        <v>-61.19999999999982</v>
       </c>
       <c r="E6">
-        <v>2776.2</v>
+        <v>2745.7</v>
       </c>
       <c r="F6">
-        <v>-61.19999999999982</v>
+        <v>-30.69999999999982</v>
       </c>
       <c r="G6">
+        <v>2646.350774298132</v>
+      </c>
+      <c r="H6">
+        <v>68.64922570186809</v>
+      </c>
+      <c r="I6">
         <v>2625.2</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>89.80000000000018</v>
       </c>
-      <c r="I6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="K6">
+        <v>2632.4</v>
+      </c>
+      <c r="L6">
+        <v>82.59999999999991</v>
+      </c>
+      <c r="M6">
+        <v>2721.6</v>
+      </c>
+      <c r="N6">
+        <v>-6.599999999999909</v>
+      </c>
+      <c r="O6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="2">
         <v>46090</v>
       </c>
@@ -596,28 +731,46 @@
         <v>2332</v>
       </c>
       <c r="C7">
-        <v>2752.87151602496</v>
+        <v>3001.6</v>
       </c>
       <c r="D7">
-        <v>-420.8715160249603</v>
+        <v>-669.5999999999999</v>
       </c>
       <c r="E7">
-        <v>3001.6</v>
+        <v>2863.5</v>
       </c>
       <c r="F7">
-        <v>-669.5999999999999</v>
+        <v>-531.5</v>
       </c>
       <c r="G7">
+        <v>2698.9916919295</v>
+      </c>
+      <c r="H7">
+        <v>-366.9916919294997</v>
+      </c>
+      <c r="I7">
         <v>2658.7</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>-326.6999999999998</v>
       </c>
-      <c r="I7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+      <c r="K7">
+        <v>2915.9</v>
+      </c>
+      <c r="L7">
+        <v>-583.9000000000001</v>
+      </c>
+      <c r="M7">
+        <v>2711.7</v>
+      </c>
+      <c r="N7">
+        <v>-379.6999999999998</v>
+      </c>
+      <c r="O7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="2">
         <v>46091</v>
       </c>
@@ -625,28 +778,46 @@
         <v>2823</v>
       </c>
       <c r="C8">
-        <v>2639.318212484806</v>
+        <v>2678.2</v>
       </c>
       <c r="D8">
-        <v>183.6817875151937</v>
+        <v>144.8000000000002</v>
       </c>
       <c r="E8">
-        <v>2678.2</v>
+        <v>2702.5</v>
       </c>
       <c r="F8">
-        <v>144.8000000000002</v>
+        <v>120.5</v>
       </c>
       <c r="G8">
+        <v>2554.027302773527</v>
+      </c>
+      <c r="H8">
+        <v>268.9726972264725</v>
+      </c>
+      <c r="I8">
         <v>2720.4</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>102.5999999999999</v>
       </c>
-      <c r="I8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="K8">
+        <v>2605.5</v>
+      </c>
+      <c r="L8">
+        <v>217.5</v>
+      </c>
+      <c r="M8">
+        <v>2652.3</v>
+      </c>
+      <c r="N8">
+        <v>170.6999999999998</v>
+      </c>
+      <c r="O8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="2">
         <v>46092</v>
       </c>
@@ -654,28 +825,46 @@
         <v>2989</v>
       </c>
       <c r="C9">
-        <v>2698.069071930044</v>
+        <v>2634.3</v>
       </c>
       <c r="D9">
-        <v>290.9309280699558</v>
+        <v>354.6999999999998</v>
       </c>
       <c r="E9">
-        <v>2634.3</v>
+        <v>2732.1</v>
       </c>
       <c r="F9">
-        <v>354.6999999999998</v>
+        <v>256.9000000000001</v>
       </c>
       <c r="G9">
+        <v>2655.333293466788</v>
+      </c>
+      <c r="H9">
+        <v>333.6667065332122</v>
+      </c>
+      <c r="I9">
         <v>2669.2</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>319.8000000000002</v>
       </c>
-      <c r="I9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="K9">
+        <v>2691</v>
+      </c>
+      <c r="L9">
+        <v>298</v>
+      </c>
+      <c r="M9">
+        <v>2687.4</v>
+      </c>
+      <c r="N9">
+        <v>301.5999999999999</v>
+      </c>
+      <c r="O9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="2">
         <v>46093</v>
       </c>
@@ -683,28 +872,46 @@
         <v>2975</v>
       </c>
       <c r="C10">
-        <v>2788.197163939301</v>
+        <v>3046.9</v>
       </c>
       <c r="D10">
-        <v>186.8028360606986</v>
+        <v>-71.90000000000009</v>
       </c>
       <c r="E10">
-        <v>3046.9</v>
+        <v>3057.5</v>
       </c>
       <c r="F10">
-        <v>-71.90000000000009</v>
+        <v>-82.5</v>
       </c>
       <c r="G10">
+        <v>2810.881330374244</v>
+      </c>
+      <c r="H10">
+        <v>164.1186696257555</v>
+      </c>
+      <c r="I10">
         <v>3268.2</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>-293.1999999999998</v>
       </c>
-      <c r="I10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="K10">
+        <v>2992.9</v>
+      </c>
+      <c r="L10">
+        <v>-17.90000000000009</v>
+      </c>
+      <c r="M10">
+        <v>3226</v>
+      </c>
+      <c r="N10">
+        <v>-251</v>
+      </c>
+      <c r="O10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="2">
         <v>46094</v>
       </c>
@@ -712,28 +919,46 @@
         <v>2985</v>
       </c>
       <c r="C11">
-        <v>2835.645498859018</v>
+        <v>3023.9</v>
       </c>
       <c r="D11">
-        <v>149.3545011409824</v>
+        <v>-38.90000000000009</v>
       </c>
       <c r="E11">
-        <v>3023.9</v>
+        <v>2992.1</v>
       </c>
       <c r="F11">
-        <v>-38.90000000000009</v>
+        <v>-7.099999999999909</v>
       </c>
       <c r="G11">
+        <v>2856.999422217285</v>
+      </c>
+      <c r="H11">
+        <v>128.0005777827155</v>
+      </c>
+      <c r="I11">
         <v>2720.4</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>264.5999999999999</v>
       </c>
-      <c r="I11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+      <c r="K11">
+        <v>3009.6</v>
+      </c>
+      <c r="L11">
+        <v>-24.59999999999991</v>
+      </c>
+      <c r="M11">
+        <v>3067.7</v>
+      </c>
+      <c r="N11">
+        <v>-82.69999999999982</v>
+      </c>
+      <c r="O11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" s="2">
         <v>46097</v>
       </c>
@@ -741,28 +966,46 @@
         <v>2905</v>
       </c>
       <c r="C12">
-        <v>2914.91444826001</v>
+        <v>2852.3</v>
       </c>
       <c r="D12">
-        <v>-9.914448260009522</v>
+        <v>52.69999999999982</v>
       </c>
       <c r="E12">
-        <v>2852.3</v>
+        <v>2881.4</v>
       </c>
       <c r="F12">
-        <v>52.69999999999982</v>
+        <v>23.59999999999991</v>
       </c>
       <c r="G12">
+        <v>2932.344420776164</v>
+      </c>
+      <c r="H12">
+        <v>-27.34442077616404</v>
+      </c>
+      <c r="I12">
         <v>2851.2</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>53.80000000000018</v>
       </c>
-      <c r="I12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="K12">
+        <v>2966.7</v>
+      </c>
+      <c r="L12">
+        <v>-61.69999999999982</v>
+      </c>
+      <c r="M12">
+        <v>2975.4</v>
+      </c>
+      <c r="N12">
+        <v>-70.40000000000009</v>
+      </c>
+      <c r="O12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="2">
         <v>46098</v>
       </c>
@@ -770,28 +1013,46 @@
         <v>3098</v>
       </c>
       <c r="C13">
-        <v>2885.837009420895</v>
+        <v>2867</v>
       </c>
       <c r="D13">
-        <v>212.1629905791051</v>
+        <v>231</v>
       </c>
       <c r="E13">
-        <v>2867</v>
+        <v>2860.4</v>
       </c>
       <c r="F13">
-        <v>231</v>
+        <v>237.5999999999999</v>
       </c>
       <c r="G13">
+        <v>2878.334908903025</v>
+      </c>
+      <c r="H13">
+        <v>219.6650910969747</v>
+      </c>
+      <c r="I13">
         <v>2848.2</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>249.8000000000002</v>
       </c>
-      <c r="I13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="K13">
+        <v>2987.2</v>
+      </c>
+      <c r="L13">
+        <v>110.8000000000002</v>
+      </c>
+      <c r="M13">
+        <v>3243.8</v>
+      </c>
+      <c r="N13">
+        <v>-145.8000000000002</v>
+      </c>
+      <c r="O13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="2">
         <v>46099</v>
       </c>
@@ -799,28 +1060,46 @@
         <v>2752</v>
       </c>
       <c r="C14">
-        <v>2932.876090968893</v>
+        <v>2997.7</v>
       </c>
       <c r="D14">
-        <v>-180.8760909688931</v>
+        <v>-245.6999999999998</v>
       </c>
       <c r="E14">
-        <v>2997.7</v>
+        <v>3006.2</v>
       </c>
       <c r="F14">
-        <v>-245.6999999999998</v>
+        <v>-254.1999999999998</v>
       </c>
       <c r="G14">
+        <v>2962.65570413351</v>
+      </c>
+      <c r="H14">
+        <v>-210.6557041335104</v>
+      </c>
+      <c r="I14">
         <v>3203.3</v>
       </c>
-      <c r="H14">
+      <c r="J14">
         <v>-451.3000000000002</v>
       </c>
-      <c r="I14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="K14">
+        <v>2989.2</v>
+      </c>
+      <c r="L14">
+        <v>-237.1999999999998</v>
+      </c>
+      <c r="M14">
+        <v>3041.1</v>
+      </c>
+      <c r="N14">
+        <v>-289.0999999999999</v>
+      </c>
+      <c r="O14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="2">
         <v>46100</v>
       </c>
@@ -828,28 +1107,46 @@
         <v>3260</v>
       </c>
       <c r="C15">
-        <v>2882.901862344557</v>
+        <v>2946.2</v>
       </c>
       <c r="D15">
-        <v>377.0981376554432</v>
+        <v>313.8000000000002</v>
       </c>
       <c r="E15">
-        <v>2946.2</v>
+        <v>2945.9</v>
       </c>
       <c r="F15">
-        <v>313.8000000000002</v>
+        <v>314.0999999999999</v>
       </c>
       <c r="G15">
+        <v>2867.958629469828</v>
+      </c>
+      <c r="H15">
+        <v>392.0413705301717</v>
+      </c>
+      <c r="I15">
         <v>2748.2</v>
       </c>
-      <c r="H15">
+      <c r="J15">
         <v>511.8000000000002</v>
       </c>
-      <c r="I15" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="K15">
+        <v>2821.4</v>
+      </c>
+      <c r="L15">
+        <v>438.5999999999999</v>
+      </c>
+      <c r="M15">
+        <v>2952</v>
+      </c>
+      <c r="N15">
+        <v>308</v>
+      </c>
+      <c r="O15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="2">
         <v>46101</v>
       </c>
@@ -857,28 +1154,46 @@
         <v>2929</v>
       </c>
       <c r="C16">
-        <v>2986.855724561461</v>
+        <v>2994.2</v>
       </c>
       <c r="D16">
-        <v>-57.8557245614611</v>
+        <v>-65.19999999999982</v>
       </c>
       <c r="E16">
-        <v>2994.2</v>
+        <v>2934</v>
       </c>
       <c r="F16">
-        <v>-65.19999999999982</v>
+        <v>-5</v>
       </c>
       <c r="G16">
+        <v>3049.945874168236</v>
+      </c>
+      <c r="H16">
+        <v>-120.9458741682361</v>
+      </c>
+      <c r="I16">
         <v>3203.3</v>
       </c>
-      <c r="H16">
+      <c r="J16">
         <v>-274.3000000000002</v>
       </c>
-      <c r="I16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="K16">
+        <v>3076.5</v>
+      </c>
+      <c r="L16">
+        <v>-147.5</v>
+      </c>
+      <c r="M16">
+        <v>3025.1</v>
+      </c>
+      <c r="N16">
+        <v>-96.09999999999991</v>
+      </c>
+      <c r="O16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" s="2">
         <v>46104</v>
       </c>
@@ -886,28 +1201,46 @@
         <v>2958</v>
       </c>
       <c r="C17">
-        <v>2995.833871821599</v>
+        <v>2833.9</v>
       </c>
       <c r="D17">
-        <v>-37.83387182159913</v>
+        <v>124.0999999999999</v>
       </c>
       <c r="E17">
-        <v>2833.9</v>
+        <v>2940.1</v>
       </c>
       <c r="F17">
-        <v>124.0999999999999</v>
+        <v>17.90000000000009</v>
       </c>
       <c r="G17">
+        <v>2990.280603733589</v>
+      </c>
+      <c r="H17">
+        <v>-32.28060373358903</v>
+      </c>
+      <c r="I17">
         <v>2836.1</v>
       </c>
-      <c r="H17">
+      <c r="J17">
         <v>121.9000000000001</v>
       </c>
-      <c r="I17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="K17">
+        <v>2920</v>
+      </c>
+      <c r="L17">
+        <v>38</v>
+      </c>
+      <c r="M17">
+        <v>2964.1</v>
+      </c>
+      <c r="N17">
+        <v>-6.099999999999909</v>
+      </c>
+      <c r="O17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" s="2">
         <v>46105</v>
       </c>
@@ -915,28 +1248,46 @@
         <v>3246</v>
       </c>
       <c r="C18">
-        <v>2947.650971999247</v>
+        <v>2885.5</v>
       </c>
       <c r="D18">
-        <v>298.3490280007527</v>
+        <v>360.5</v>
       </c>
       <c r="E18">
-        <v>2885.5</v>
+        <v>2893.9</v>
       </c>
       <c r="F18">
-        <v>360.5</v>
+        <v>352.0999999999999</v>
       </c>
       <c r="G18">
+        <v>2970.132821424485</v>
+      </c>
+      <c r="H18">
+        <v>275.867178575515</v>
+      </c>
+      <c r="I18">
         <v>2875.9</v>
       </c>
-      <c r="H18">
+      <c r="J18">
         <v>370.0999999999999</v>
       </c>
-      <c r="I18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="K18">
+        <v>2942.9</v>
+      </c>
+      <c r="L18">
+        <v>303.0999999999999</v>
+      </c>
+      <c r="M18">
+        <v>2985.1</v>
+      </c>
+      <c r="N18">
+        <v>260.9000000000001</v>
+      </c>
+      <c r="O18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" s="2">
         <v>46106</v>
       </c>
@@ -944,28 +1295,46 @@
         <v>3142</v>
       </c>
       <c r="C19">
-        <v>3053.390972620517</v>
+        <v>2946.5</v>
       </c>
       <c r="D19">
-        <v>88.609027379483</v>
+        <v>195.5</v>
       </c>
       <c r="E19">
-        <v>2946.5</v>
+        <v>3004.8</v>
       </c>
       <c r="F19">
-        <v>195.5</v>
+        <v>137.1999999999998</v>
       </c>
       <c r="G19">
+        <v>3108.959524377238</v>
+      </c>
+      <c r="H19">
+        <v>33.04047562276173</v>
+      </c>
+      <c r="I19">
         <v>3119.2</v>
       </c>
-      <c r="H19">
+      <c r="J19">
         <v>22.80000000000018</v>
       </c>
-      <c r="I19" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="K19">
+        <v>2953.7</v>
+      </c>
+      <c r="L19">
+        <v>188.3000000000002</v>
+      </c>
+      <c r="M19">
+        <v>3044.4</v>
+      </c>
+      <c r="N19">
+        <v>97.59999999999991</v>
+      </c>
+      <c r="O19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" s="2">
         <v>46107</v>
       </c>
@@ -973,28 +1342,46 @@
         <v>3002</v>
       </c>
       <c r="C20">
-        <v>3042.326969786985</v>
+        <v>3085.9</v>
       </c>
       <c r="D20">
-        <v>-40.32696978698505</v>
+        <v>-83.90000000000009</v>
       </c>
       <c r="E20">
-        <v>3085.9</v>
+        <v>3032.4</v>
       </c>
       <c r="F20">
-        <v>-83.90000000000009</v>
+        <v>-30.40000000000009</v>
       </c>
       <c r="G20">
+        <v>3093.601759111588</v>
+      </c>
+      <c r="H20">
+        <v>-91.60175911158785</v>
+      </c>
+      <c r="I20">
         <v>3028.9</v>
       </c>
-      <c r="H20">
+      <c r="J20">
         <v>-26.90000000000009</v>
       </c>
-      <c r="I20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="K20">
+        <v>3116.1</v>
+      </c>
+      <c r="L20">
+        <v>-114.0999999999999</v>
+      </c>
+      <c r="M20">
+        <v>3004.3</v>
+      </c>
+      <c r="N20">
+        <v>-2.300000000000182</v>
+      </c>
+      <c r="O20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" s="2">
         <v>46108</v>
       </c>
@@ -1002,28 +1389,46 @@
         <v>3322</v>
       </c>
       <c r="C21">
-        <v>3054.194158411876</v>
+        <v>3145.4</v>
       </c>
       <c r="D21">
-        <v>267.8058415881237</v>
+        <v>176.5999999999999</v>
       </c>
       <c r="E21">
-        <v>3145.4</v>
+        <v>3053.1</v>
       </c>
       <c r="F21">
-        <v>176.5999999999999</v>
+        <v>268.9000000000001</v>
       </c>
       <c r="G21">
+        <v>3079.229224385529</v>
+      </c>
+      <c r="H21">
+        <v>242.7707756144709</v>
+      </c>
+      <c r="I21">
         <v>3054.8</v>
       </c>
-      <c r="H21">
+      <c r="J21">
         <v>267.1999999999998</v>
       </c>
-      <c r="I21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="K21">
+        <v>3240.4</v>
+      </c>
+      <c r="L21">
+        <v>81.59999999999991</v>
+      </c>
+      <c r="M21">
+        <v>3085</v>
+      </c>
+      <c r="N21">
+        <v>237</v>
+      </c>
+      <c r="O21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" s="2">
         <v>46111</v>
       </c>
@@ -1031,28 +1436,46 @@
         <v>3279</v>
       </c>
       <c r="C22">
-        <v>3139.949555679771</v>
+        <v>2905.7</v>
       </c>
       <c r="D22">
-        <v>139.0504443202294</v>
+        <v>373.3000000000002</v>
       </c>
       <c r="E22">
-        <v>2905.7</v>
+        <v>2933.1</v>
       </c>
       <c r="F22">
-        <v>373.3000000000002</v>
+        <v>345.9000000000001</v>
       </c>
       <c r="G22">
+        <v>3183.303165557737</v>
+      </c>
+      <c r="H22">
+        <v>95.69683444226348</v>
+      </c>
+      <c r="I22">
         <v>2831.3</v>
       </c>
-      <c r="H22">
+      <c r="J22">
         <v>447.6999999999998</v>
       </c>
-      <c r="I22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+      <c r="K22">
+        <v>2862.2</v>
+      </c>
+      <c r="L22">
+        <v>416.8000000000002</v>
+      </c>
+      <c r="M22">
+        <v>2910.8</v>
+      </c>
+      <c r="N22">
+        <v>368.1999999999998</v>
+      </c>
+      <c r="O22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15">
       <c r="A23" s="2">
         <v>46112</v>
       </c>
@@ -1060,25 +1483,43 @@
         <v>2935</v>
       </c>
       <c r="C23">
-        <v>3146.209939922689</v>
+        <v>3017.2</v>
       </c>
       <c r="D23">
-        <v>-211.209939922689</v>
+        <v>-82.19999999999982</v>
       </c>
       <c r="E23">
-        <v>3017.2</v>
+        <v>3034</v>
       </c>
       <c r="F23">
-        <v>-82.19999999999982</v>
+        <v>-99</v>
       </c>
       <c r="G23">
+        <v>3211.580154655469</v>
+      </c>
+      <c r="H23">
+        <v>-276.5801546554685</v>
+      </c>
+      <c r="I23">
         <v>3054.8</v>
       </c>
-      <c r="H23">
+      <c r="J23">
         <v>-119.8000000000002</v>
       </c>
-      <c r="I23" t="s">
-        <v>9</v>
+      <c r="K23">
+        <v>3053.6</v>
+      </c>
+      <c r="L23">
+        <v>-118.5999999999999</v>
+      </c>
+      <c r="M23">
+        <v>3007.9</v>
+      </c>
+      <c r="N23">
+        <v>-72.90000000000009</v>
+      </c>
+      <c r="O23" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>